<commit_message>
배포판 자동 동기화 — 3ca933b (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -455,9 +455,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -465,9 +463,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -475,9 +471,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -485,9 +479,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -495,9 +487,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -505,9 +495,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -515,9 +503,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -560,9 +546,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -626,9 +610,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -810,7 +792,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>이름01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -833,7 +815,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>이름02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -856,7 +838,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>이름03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -879,7 +861,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>이름04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -902,7 +884,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>이름05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -930,7 +912,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>이름06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -953,7 +935,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>이름07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -976,7 +958,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>이름08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -999,7 +981,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>이름09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1022,7 +1004,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>이름10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1050,7 +1032,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>이름11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1073,7 +1055,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>이름12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1101,7 +1083,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>이름13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1129,7 +1111,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>이름14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1152,7 +1134,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>이름15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1175,7 +1157,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>이름16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1198,7 +1180,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>이름17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1221,7 +1203,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>이름18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1244,7 +1226,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>이름19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1267,7 +1249,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>이름20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1290,7 +1272,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>이름21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1313,7 +1295,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>이름22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1336,7 +1318,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>이름23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1359,7 +1341,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>이름24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1382,7 +1364,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>이름25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1405,7 +1387,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>이름26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1428,7 +1410,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>이름27</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1451,7 +1433,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>이름28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1474,7 +1456,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>이름29</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1497,7 +1479,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>이름30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1520,7 +1502,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>이름31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1543,7 +1525,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>이름32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1566,7 +1548,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>이름33</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1589,7 +1571,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>이름34</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1612,7 +1594,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>이름35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1635,7 +1617,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>이름36</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1658,7 +1640,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>이름37</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1681,7 +1663,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>이름38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1704,7 +1686,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>이름39</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1727,7 +1709,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>파트장</t>
+          <t>파트장이름</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1757,14 +1739,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>이름40</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>이름41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 7a1cabd (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -455,7 +455,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -463,7 +462,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -471,7 +469,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -479,7 +476,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -487,7 +483,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -495,7 +490,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -503,7 +497,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -546,7 +539,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -610,7 +602,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -792,12 +783,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>이름01</t>
+          <t>파트장이름</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>간호사</t>
+          <t>파트장</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -807,7 +798,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>8A</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -815,7 +806,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>이름02</t>
+          <t>이름01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -838,7 +829,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>이름03</t>
+          <t>이름02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -853,7 +844,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -861,7 +852,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>이름04</t>
+          <t>이름03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -876,7 +867,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>prn</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -884,7 +875,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>이름05</t>
+          <t>이름04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -899,12 +890,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D,E</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>임부(야간 금지)</t>
+          <t>prn</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -912,7 +898,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>이름06</t>
+          <t>이름05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -927,7 +913,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>임부(야간 금지)</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -935,7 +926,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>이름07</t>
+          <t>이름06</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -958,7 +949,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>이름08</t>
+          <t>이름07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -981,7 +972,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>이름09</t>
+          <t>이름08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1004,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>이름10</t>
+          <t>이름09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1019,12 +1010,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NK</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>야간전담</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
@@ -1032,7 +1018,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>이름11</t>
+          <t>이름10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1047,7 +1033,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>야간전담</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -1055,7 +1046,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>이름12</t>
+          <t>이름11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1065,17 +1056,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lv4</t>
+          <t>Lv5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NK</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>야간전담</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
@@ -1083,7 +1069,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>이름13</t>
+          <t>이름12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1098,12 +1084,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>D,E</t>
+          <t>NK</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>임부(야간 금지)</t>
+          <t>야간전담</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -1111,7 +1097,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>이름14</t>
+          <t>이름13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1121,12 +1107,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Lv3</t>
+          <t>Lv4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>D,E</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>임부(야간 금지)</t>
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
@@ -1134,7 +1125,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>이름15</t>
+          <t>이름14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1149,7 +1140,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1157,7 +1148,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>이름16</t>
+          <t>이름15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1172,7 +1163,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
@@ -1180,7 +1171,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>이름17</t>
+          <t>이름16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1195,7 +1186,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1203,7 +1194,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>이름18</t>
+          <t>이름17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1226,7 +1217,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>이름19</t>
+          <t>이름18</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1236,7 +1227,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lv2</t>
+          <t>Lv3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1249,7 +1240,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>이름20</t>
+          <t>이름19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1259,7 +1250,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Lv3</t>
+          <t>Lv2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1272,7 +1263,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>이름21</t>
+          <t>이름20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1282,7 +1273,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lv2</t>
+          <t>Lv3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1295,7 +1286,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>이름22</t>
+          <t>이름21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1305,7 +1296,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Lv3</t>
+          <t>Lv2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1318,7 +1309,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>이름23</t>
+          <t>이름22</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1333,7 +1324,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1341,7 +1332,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>이름24</t>
+          <t>이름23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1356,7 +1347,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
@@ -1364,7 +1355,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>이름25</t>
+          <t>이름24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1387,7 +1378,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>이름26</t>
+          <t>이름25</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1410,7 +1401,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>이름27</t>
+          <t>이름26</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1420,7 +1411,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lv2</t>
+          <t>Lv3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1433,7 +1424,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>이름28</t>
+          <t>이름27</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1456,7 +1447,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>이름29</t>
+          <t>이름28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1479,7 +1470,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>이름30</t>
+          <t>이름29</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1502,7 +1493,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>이름31</t>
+          <t>이름30</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1517,7 +1508,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G34" s="2" t="n"/>
@@ -1525,7 +1516,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>이름32</t>
+          <t>이름31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1540,7 +1531,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,prn</t>
         </is>
       </c>
       <c r="G35" s="2" t="n"/>
@@ -1548,7 +1539,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>이름33</t>
+          <t>이름32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1571,7 +1562,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>이름34</t>
+          <t>이름33</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1594,7 +1585,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>이름35</t>
+          <t>이름34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1617,7 +1608,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>이름36</t>
+          <t>이름35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1627,7 +1618,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lv1</t>
+          <t>Lv2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1640,7 +1631,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>이름37</t>
+          <t>이름36</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1663,7 +1654,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>이름38</t>
+          <t>이름37</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1686,7 +1677,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>이름39</t>
+          <t>이름38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1709,22 +1700,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>파트장이름</t>
+          <t>이름39</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>파트장</t>
+          <t>간호사</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Lv5</t>
+          <t>Lv1</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>8A</t>
+          <t>D,E,N</t>
         </is>
       </c>
       <c r="G43" s="2" t="n"/>

</xml_diff>

<commit_message>
배포판 자동 동기화 — f4736a0 (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -821,7 +821,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,지정</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,지정</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -867,7 +867,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N,prn,3N</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -941,7 +941,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,2N</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 1f5e8ff (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -1186,7 +1186,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>D,E,N,prn</t>
+          <t>D,E,N,prn,지정</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,지정</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>D,E,N</t>
+          <t>D,E,N,지정</t>
         </is>
       </c>
       <c r="G32" s="2" t="n"/>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 82368cd (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력1_원티드표_샘플.xlsx
+++ b/templates/입력1_원티드표_샘플.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,9 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -462,6 +465,9 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -469,148 +475,196 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>⚠ '전입'·'전입일' 칸 — 이번 달에 새로 온 사람은 '전입'을 고르고, 월중 입사면 입사일을 적어주세요(비우면 1일자 전입). 입사 전 날짜는 배정에서 빠집니다.</t>
-        </is>
-      </c>
+          <t>⚠ '가능근무' 칸에는 근무코드(D·E·N·prn 등) 외에 세 가지를 더 적을 수 있습니다. 2N·3N은 야간을 며칠씩 묶어 서고 싶은지입니다(안 적으면 2N). 3N은 3일씩 묶어 서므로 그 사람의 월 야간이 상한(기본 6회)으로 고정됩니다 — 3일 블록으로는 하한 4를 만들 수 없기 때문입니다. '지정'은 근무인력 표의 '지정' 인원으로 셀 수 있는 사람이라는 표시로, 그날 D·E·N·prn 중 무엇이든 서면 자동으로 한 명으로 세집니다. 셋 다 근무가 아니라 표시라서, D·E·N 같은 근무를 함께 적어야 배정됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>⚠ 날짜 칸은 OCS 화면에서 그대로 복사해 붙여넣어도 됩니다 — 말일 칸 오른쪽에 딸려온 D/E/N·®·ⓡ·금월·T연·R연·부서 같은 칸은 읽지 않으니 그냥 두셔도 되고 지우셔도 됩니다.</t>
-        </is>
-      </c>
+          <t>⚠ prn 인원은 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8A◎ 등)을 한 덩어리로 셉니다 — 시작 시각만 다른 같은 근무라서입니다. 반일 근무(8AH·9AH·9H*)만 0.5명으로 세기 때문에 출력 근무표의 'prn 인원' 줄에 2.5 같은 값이 뜰 수 있습니다(반나절 선 사람을 온종일 선 것으로 세면 못 채운 날이 채운 날처럼 보이기 때문입니다).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>⚠ 인원 명단 아래 이름 칸에 'B' 한 글자만 있는 구분 행과 그 아래 이름들은 B팀(신입)입니다 — 근무 배정에는 전혀 관여하지 않고 출력 근무표에 이름만 표시됩니다. 필요 없으면 그 행들을 지우고 올리세요.</t>
-        </is>
-      </c>
+          <t>⚠ '전입'·'전입일' 칸 — 이번 달에 새로 온 사람은 '전입'을 고르고, 월중 입사면 입사일을 적어주세요(비우면 1일자 전입). 입사 전 날짜는 배정에서 빠집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>⚠ 중요 — '원티드표' 시트의 A1 셀에 적힌 'YYYY년 M월'을 보고 코드가 이 파일이 몇 년 몇 월 신청분인지 자동으로 인식합니다. A1의 월 이름을 실제 신청 대상 월과 다르게 고치면(예: 파일을 복사해서 재사용하다가 안 고침) 엉뚱한 달로 인식되니, 월을 바꿀 때는 A1도 꼭 같이 맞춰주세요 — 파일명이 아니라 A1 셀 내용을 봅니다.</t>
-        </is>
-      </c>
+          <t>⚠ 날짜 칸은 OCS 화면에서 그대로 복사해 붙여넣어도 됩니다 — 말일 칸 오른쪽에 딸려온 D/E/N·®·ⓡ·금월·T연·R연·부서 같은 칸은 읽지 않으니 그냥 두셔도 되고 지우셔도 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>표기 코드 (뒤에 별표 * 가 있어도 없어도 인식됩니다)</t>
+          <t>⚠ 인원 명단 아래 이름 칸에 'B' 한 글자만 있는 구분 행과 그 아래 이름들은 B팀(신입)입니다 — 근무 배정에는 전혀 관여하지 않고 출력 근무표에 이름만 표시됩니다. 필요 없으면 그 행들을 지우고 올리세요.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>· 근무 희망: D / E / N / 8A / 9A / NK / prn / T(교육) / TW(반근무+반교육)</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>· 휴가유형별 희망: 연·연차(연차) / 연1·연2·연3(시간제 연차) / 연4(반차) / 조(조사) / 경(경조사) / 공(공가) / 병(병가) / 휴(휴직) / 승(승급교육) / 군(군공가) / S/(수면오프)</t>
+          <t>⚠ 중요 — '원티드표' 시트의 A1 셀에 적힌 'YYYY년 M월'을 보고 코드가 이 파일이 몇 년 몇 월 신청분인지 자동으로 인식합니다. A1의 월 이름을 실제 신청 대상 월과 다르게 고치면(예: 파일을 복사해서 재사용하다가 안 고침) 엉뚱한 달로 인식되니, 월을 바꿀 때는 A1도 꼭 같이 맞춰주세요 — 파일명이 아니라 A1 셀 내용을 봅니다.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>· 단순 OFF 희망: X</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>· 그 외 인식 못 하는 표시(포상휴가 등 특수 코드)는 업로드 후 '인식 못 한 표시' 목록으로 알려드립니다.</t>
+          <t>표기 코드 (뒤에 별표 * 가 있어도 없어도 인식됩니다)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>· 빈 칸은 신청 없음으로 건너뜁니다.</t>
+          <t>· 근무 희망: D / E / N / 8A / 9A / NK / prn / T(교육) / TW(반근무+반교육)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>· 휴가유형별 희망: 연·연차(연차) / 연1·연2·연3(시간제 연차) / 연4(반차) / 조(조사) / 경(경조사) / 공(공가) / 병(병가) / 휴(휴직) / 승(승급교육) / 군(군공가)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>각 코드가 배정에서 어떻게 처리되는지</t>
+          <t>· 단순 OFF 희망: X</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>· 병(병가): 연속근무일수 계산에서 제외됩니다(연속근무 5일 제한에 안 걸림)</t>
+          <t>· 그 외 인식 못 하는 표시(포상휴가 등 특수 코드)는 업로드 후 '인식 못 한 표시' 목록으로 알려드립니다.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>· 휴(휴직): 신청일부터 그 달 나머지 기간 전부 휴직으로 자동 처리됩니다</t>
+          <t>· 빈 칸은 신청 없음으로 건너뜁니다.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>· 공/승(공가/승급교육): 휴무(OFF)와 동일하게 취급되지만 연차는 차감되지 않습니다</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>· 연1/연2/연3/연4(시간제/반차 연차): 몇 시간이든 하루치 연차 희망으로 집계됩니다</t>
+          <t>각 코드가 배정에서 어떻게 처리되는지</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>· 군(군공가)/S/(수면오프): 휴무(OFF)와 동일하게 취급되지만 잔휴에는 반영되지 않습니다</t>
+          <t>· 병(병가): 연속근무일수 계산에서 제외됩니다(연속근무 5일 제한에 안 걸림)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>· S/(수면오프)는 월 야간이 6회 이상이면 프로그램이 오프 하루를 S/로 바꿔 자동으로 넣어줍니다 — 따로 신청하지 않아도 됩니다(그 달 안에서 날짜는 자유롭게 옮겨 쓰세요)</t>
+          <t>· 휴(휴직): **적은 날짜 하루만** 제외됩니다. 월 나머지가 자동으로 채워지지 않으니 휴직·장기휴가는 쉬는 날마다 한 칸씩 적어주세요(며칠짜리인지는 파트장이 지정).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>· TW(반근무+반교육): 근무일수엔 포함되지만 최소인력 계산에는 제외됩니다(교육 T와 동일)</t>
+          <t xml:space="preserve">  같은 방식으로 사(사사휴직)/상(상병휴직)/산전/육법/육연/R/출산도 날짜마다 적습니다.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>· 9A(09시 시작): 8A와 동격으로 취급됩니다(시작 시각만 다름)</t>
+          <t>· 공/승(공가/승급교육): 휴무(OFF)와 동일하게 취급되지만 연차는 차감되지 않습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>· 연1/연2/연3/연4(시간제/반차 연차): 몇 시간이든 하루치 연차 희망으로 집계됩니다</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>가장 쉬운 사용법</t>
+          <t>· 군(군공가): 휴무(OFF)와 동일하게 취급되지만 잔휴에는 반영되지 않습니다</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
+        <is>
+          <t>· S/(수면오프)는 이 표에 신청할 수 없습니다 — 월 야간이 6회 이상이면 프로그램이 자동으로 하루 넣어줍니다. 오프를 대신 쓰는 것이 아니라 오프와 별도로 하루가 더 생깁니다(그 달 안에서 날짜는 자유롭게 옮겨 쓰세요). 야간이 몇 회든 1개이고, 원티드로는 신청할 수 없습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>· TW(반근무+반교육): 근무일수엔 포함되지만 최소인력 계산에는 제외됩니다(교육 T와 동일)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>· 9A(09시 시작): 8A와 동격으로 취급됩니다(시작 시각만 다름). 8A·9A·10A와 8H·9H·10H, 그리고 그 변형(8A*·8AH 등)은 하단 'prn 인원'에 함께 잡힙니다 — 반일 근무(8AH·9AH·9H*)만 0.5명으로 셉니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>가장 쉬운 사용법</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>이번 달 근무표를 아무 값이나 넣어 한 번 생성해서 빈 그리드 모양(입력②와 같은 모양)을 받은 뒤, 그 위에 표시만 채워서 다시 올려도 됩니다.</t>
         </is>

</xml_diff>